<commit_message>
Update artifact templates, examples, and manifest
Sync the latest FORM templates and worked-example documents, including
newly added artifacts, and update the template manifest to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/examples/A-003-MasterAssetInventory-EXAMPLE-L.xlsx
+++ b/public/templates/examples/A-003-MasterAssetInventory-EXAMPLE-L.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="0"/>
   <fonts count="8">
     <font>
-      <name val="Calibri"/>
+      <name val="Aptos"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -224,12 +224,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="552450" cy="552450"/>
+    <ext cx="857250" cy="857250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -393,7 +393,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Aptos"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -427,7 +427,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>

</xml_diff>

<commit_message>
Complete corpus (163 forms, 489 examples); curate ambiguous brackets and acronym labels
Library: the full authored corpus is now in the repo — 100 docx + 63 xlsx forms,
489 worked examples, with regenerated traceability, manifest, and compiled copies.
Tracker renamed off the "--" prefix; generate-lookup and related data updated.

Curation against the complete corpus:
- Ambiguous brackets 45 -> 0: 2 dropdowns (Severity, Remote-Access Method), 14
  fill-in fields, 29 complete-default/cross-reference statements un-bracketed to
  literal, [12 months] relabeled to [review period]. A-046 outer scope bracket
  removed with its inner [Director / Coordinator] field kept.
- securityCoordinator curated as a shared, fill-once role (recurred across 15 forms).
- humanizeTag is acronym-aware (MFA, IT, CAD, NTP, SIP, CJIS, VLAN, VoIP, ESInet,
  DMZ, RTO, RPO, GIS, IDS, IPS, ...), so the un-curated tail labels correctly.

tsc / eslint / strict template-lint / next build all green.
</commit_message>
<xml_diff>
--- a/public/templates/examples/A-003-MasterAssetInventory-EXAMPLE-L.xlsx
+++ b/public/templates/examples/A-003-MasterAssetInventory-EXAMPLE-L.xlsx
@@ -4,19 +4,24 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Register!$11:$11</definedName>
+  </definedNames>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <name val="Aptos"/>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -142,6 +147,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf applyNumberFormat="1" numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyNumberFormat="1" numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -637,7 +648,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -840,7 +851,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19.5" customHeight="1">
+    <row r="12" ht="34.7" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>AST-001</t>
@@ -886,18 +897,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="19.5" customHeight="1">
+      <c r="J12" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K12" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="13" ht="34.7" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>AST-002</t>
@@ -943,18 +950,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="19.5" customHeight="1">
+      <c r="J13" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K13" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="14" ht="34.7" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>AST-003</t>
@@ -1000,18 +1003,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="19.5" customHeight="1">
+      <c r="J14" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K14" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="15" ht="34.7" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>AST-004</t>
@@ -1057,18 +1056,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
+      <c r="J15" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K15" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="16" ht="34.7" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>AST-005</t>
@@ -1114,18 +1109,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
+      <c r="J16" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K16" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="17" ht="34.7" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>AST-006</t>
@@ -1171,18 +1162,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="19.5" customHeight="1">
+      <c r="J17" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K17" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="18" ht="34.7" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>AST-007</t>
@@ -1228,18 +1215,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="19.5" customHeight="1">
+      <c r="J18" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K18" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="19" ht="34.7" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>AST-008</t>
@@ -1285,18 +1268,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="19.5" customHeight="1">
+      <c r="J19" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K19" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="20" ht="34.7" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>AST-009</t>
@@ -1342,18 +1321,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="19.5" customHeight="1">
+      <c r="J20" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K20" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="21" ht="34.7" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>AST-010</t>
@@ -1399,18 +1374,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="19.5" customHeight="1">
+      <c r="J21" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K21" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="22" ht="34.7" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>AST-011</t>
@@ -1456,18 +1427,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="19.5" customHeight="1">
+      <c r="J22" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K22" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="23" ht="34.7" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>AST-012</t>
@@ -1513,18 +1480,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="19.5" customHeight="1">
+      <c r="J23" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K23" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="24" ht="34.7" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>AST-013</t>
@@ -1570,18 +1533,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="19.5" customHeight="1">
+      <c r="J24" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K24" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="25" ht="34.7" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>AST-014</t>
@@ -1627,18 +1586,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="19.5" customHeight="1">
+      <c r="J25" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K25" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="26" ht="34.7" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>AST-015</t>
@@ -1684,18 +1639,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="19.5" customHeight="1">
+      <c r="J26" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K26" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="27" ht="34.7" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>AST-016</t>
@@ -1741,18 +1692,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="19.5" customHeight="1">
+      <c r="J27" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K27" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="28" ht="34.7" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>AST-017</t>
@@ -1798,18 +1745,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K28" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="19.5" customHeight="1">
+      <c r="J28" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K28" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="29" ht="34.7" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>AST-018</t>
@@ -1855,18 +1798,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="19.5" customHeight="1">
+      <c r="J29" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K29" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="30" ht="34.7" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>AST-019</t>
@@ -1912,18 +1851,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K30" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="19.5" customHeight="1">
+      <c r="J30" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K30" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="31" ht="34.7" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>AST-020</t>
@@ -1969,18 +1904,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J31" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="19.5" customHeight="1">
+      <c r="J31" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K31" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="32" ht="34.7" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>AST-021</t>
@@ -2026,18 +1957,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J32" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K32" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="19.5" customHeight="1">
+      <c r="J32" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K32" s="14">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="33" ht="34.7" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>AST-022</t>
@@ -2083,15 +2010,11 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J33" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
+      <c r="J33" s="14">
+        <v>46078</v>
+      </c>
+      <c r="K33" s="14">
+        <v>46101</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1"/>
@@ -2139,7 +2062,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="19.5" customHeight="1">
+    <row r="37" ht="34.7" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>AST-001</t>
@@ -2165,10 +2088,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F37" s="14">
+        <v>46078</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -2176,7 +2097,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="19.5" customHeight="1">
+    <row r="38" ht="34.7" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>AST-002</t>
@@ -2202,10 +2123,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F38" s="14">
+        <v>46078</v>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
@@ -2213,7 +2132,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="19.5" customHeight="1">
+    <row r="39" ht="34.7" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>AST-004</t>
@@ -2239,10 +2158,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F39" s="14">
+        <v>46078</v>
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
@@ -2250,7 +2167,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="19.5" customHeight="1">
+    <row r="40" ht="34.7" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>AST-005</t>
@@ -2276,10 +2193,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F40" s="14">
+        <v>46078</v>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
@@ -2287,7 +2202,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="19.5" customHeight="1">
+    <row r="41" ht="34.7" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>AST-006</t>
@@ -2313,10 +2228,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F41" s="14">
+        <v>46078</v>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
@@ -2324,7 +2237,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="19.5" customHeight="1">
+    <row r="42" ht="50.5" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>AST-009</t>
@@ -2350,10 +2263,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F42" s="14">
+        <v>46078</v>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
@@ -2361,7 +2272,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="19.5" customHeight="1">
+    <row r="43" ht="50.5" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>AST-010</t>
@@ -2387,10 +2298,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F43" s="14">
+        <v>46078</v>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
@@ -2398,7 +2307,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="19.5" customHeight="1">
+    <row r="44" ht="50.5" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>AST-011</t>
@@ -2424,10 +2333,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F44" s="14">
+        <v>46078</v>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
@@ -2435,7 +2342,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="19.5" customHeight="1">
+    <row r="45" ht="50.5" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>AST-012</t>
@@ -2461,10 +2368,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F45" s="14">
+        <v>46078</v>
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2377,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="19.5" customHeight="1">
+    <row r="46" ht="50.5" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>AST-013</t>
@@ -2498,10 +2403,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F46" s="14">
+        <v>46078</v>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
@@ -2509,7 +2412,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="19.5" customHeight="1">
+    <row r="47" ht="50.5" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>AST-014</t>
@@ -2535,10 +2438,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F47" s="14">
+        <v>46078</v>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
@@ -2546,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="19.5" customHeight="1">
+    <row r="48" ht="50.5" customHeight="1">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>AST-015</t>
@@ -2572,10 +2473,8 @@
           <t>EDR agent (managed)</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
+      <c r="F48" s="14">
+        <v>46078</v>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
@@ -2587,7 +2486,7 @@
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Summary (as of 2026-03-21)</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2498,6 @@
       </c>
       <c r="C51" s="10">
         <f>COUNTA(A12:A33)</f>
-        <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
@@ -2610,7 +2508,6 @@
       </c>
       <c r="C52" s="10">
         <f>COUNTIF(I12:I33,"Active")</f>
-        <v/>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
@@ -2621,7 +2518,6 @@
       </c>
       <c r="C53" s="10">
         <f>COUNTIF(I12:I33,"Under Review")</f>
-        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
@@ -2632,7 +2528,6 @@
       </c>
       <c r="C54" s="10">
         <f>COUNTIF(I12:I33,"Retired")</f>
-        <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
@@ -2643,7 +2538,6 @@
       </c>
       <c r="C55" s="10">
         <f>COUNTIF(I12:I33,"Decommissioned")</f>
-        <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
@@ -2653,8 +2547,7 @@
         </is>
       </c>
       <c r="C56" s="10">
-        <f>COUNTIF(K12:K33,"&lt;"&amp;TODAY())</f>
-        <v/>
+        <f>COUNTIF(K12:K33,"&lt;"&amp;DATE(2026,3,21))</f>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1"/>
@@ -2740,10 +2633,8 @@
           <t>Dr. Lisa Park</t>
         </is>
       </c>
-      <c r="D67" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="D67" s="15">
+        <v>46082</v>
       </c>
     </row>
     <row r="68" ht="26" customHeight="1">
@@ -2762,10 +2653,8 @@
           <t>(on file)</t>
         </is>
       </c>
-      <c r="D68" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="D68" s="15">
+        <v>46082</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1"/>
@@ -2804,10 +2693,8 @@
           <t>3.0</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>2025-12-01</t>
-        </is>
+      <c r="B72" s="14">
+        <v>45992</v>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
@@ -2820,16 +2707,14 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="17" customHeight="1">
+    <row r="73" ht="66.4" customHeight="1">
       <c r="A73" s="8" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="B73" s="14">
+        <v>46082</v>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
@@ -2867,7 +2752,8 @@
     <mergeCell ref="A10:K10"/>
     <mergeCell ref="C4:K4"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>